<commit_message>
refactor: update insertion_sort, sellSort_base_line, experimento and resultados.xlsx
</commit_message>
<xml_diff>
--- a/docs/resultados.xlsx
+++ b/docs/resultados.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Renato\Documents\GitHub\algorithm-complexity-experiment-recursion\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DDD29F19-E9F6-45DC-993C-EC6C00187A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F27F3C47-BBDE-4776-BE6D-8A8D529DCC68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{16E4E982-502A-480D-A0DC-EBABC411A963}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{16E4E982-502A-480D-A0DC-EBABC411A963}"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="Decrescentes" sheetId="1" r:id="rId1"/>
+    <sheet name="Crescentes" sheetId="2" r:id="rId2"/>
+    <sheet name="Randômicos" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="10">
   <si>
     <t>QS1</t>
   </si>
@@ -75,8 +77,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -104,8 +114,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -440,10 +452,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B389985-64A3-4E61-9B8D-F3723E49502C}">
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -475,7 +487,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>2</v>
       </c>
@@ -483,35 +495,723 @@
         <v>0</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G2">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H2">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="I2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>8</v>
       </c>
       <c r="B3">
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>15</v>
+      </c>
+      <c r="G3">
+        <v>49</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>6</v>
+      </c>
+      <c r="J3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>19</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4">
+        <v>32</v>
+      </c>
+      <c r="G4">
+        <v>116</v>
+      </c>
+      <c r="H4">
+        <v>1</v>
+      </c>
+      <c r="I4">
+        <v>15</v>
+      </c>
+      <c r="J4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>36</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>58</v>
+      </c>
+      <c r="G5">
+        <v>224</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>28</v>
+      </c>
+      <c r="J5">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>58</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>2</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6">
+        <v>91</v>
+      </c>
+      <c r="G6">
+        <v>352</v>
+      </c>
+      <c r="H6">
+        <v>1</v>
+      </c>
+      <c r="I6">
+        <v>46</v>
+      </c>
+      <c r="J6">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>81</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7">
+        <v>131</v>
+      </c>
+      <c r="G7">
+        <v>525</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>63</v>
+      </c>
+      <c r="J7">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>108</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8">
+        <v>3</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8">
+        <v>3</v>
+      </c>
+      <c r="F8">
+        <v>180</v>
+      </c>
+      <c r="G8">
+        <v>701</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>87</v>
+      </c>
+      <c r="J8">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>144</v>
+      </c>
+      <c r="B9">
+        <v>2</v>
+      </c>
+      <c r="C9">
+        <v>3</v>
+      </c>
+      <c r="D9">
+        <v>3</v>
+      </c>
+      <c r="E9">
+        <v>3</v>
+      </c>
+      <c r="F9">
+        <v>236</v>
+      </c>
+      <c r="G9">
+        <v>940</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>120</v>
+      </c>
+      <c r="J9">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>182</v>
+      </c>
+      <c r="B10">
+        <v>4</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <v>3</v>
+      </c>
+      <c r="E10">
+        <v>4</v>
+      </c>
+      <c r="F10">
+        <v>297</v>
+      </c>
+      <c r="G10">
+        <v>1192</v>
+      </c>
+      <c r="H10">
+        <v>2</v>
+      </c>
+      <c r="I10">
+        <v>149</v>
+      </c>
+      <c r="J10">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>223</v>
+      </c>
+      <c r="B11">
+        <v>4</v>
+      </c>
+      <c r="C11">
+        <v>4</v>
+      </c>
+      <c r="D11">
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>5</v>
+      </c>
+      <c r="F11">
+        <v>367</v>
+      </c>
+      <c r="G11">
+        <v>1497</v>
+      </c>
+      <c r="H11">
+        <v>2</v>
+      </c>
+      <c r="I11">
+        <v>181</v>
+      </c>
+      <c r="J11">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>271</v>
+      </c>
+      <c r="B12">
+        <v>4</v>
+      </c>
+      <c r="C12">
+        <v>4</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <v>5</v>
+      </c>
+      <c r="F12">
+        <v>454</v>
+      </c>
+      <c r="G12">
+        <v>1872</v>
+      </c>
+      <c r="H12">
+        <v>2</v>
+      </c>
+      <c r="I12">
+        <v>220</v>
+      </c>
+      <c r="J12">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>323</v>
+      </c>
+      <c r="B13">
+        <v>4</v>
+      </c>
+      <c r="C13">
+        <v>4</v>
+      </c>
+      <c r="D13">
+        <v>4</v>
+      </c>
+      <c r="E13">
+        <v>5</v>
+      </c>
+      <c r="F13">
+        <v>525</v>
+      </c>
+      <c r="G13">
+        <v>2166</v>
+      </c>
+      <c r="H13">
+        <v>2</v>
+      </c>
+      <c r="I13">
+        <v>265</v>
+      </c>
+      <c r="J13">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>391</v>
+      </c>
+      <c r="B14">
+        <v>5</v>
+      </c>
+      <c r="C14">
+        <v>5</v>
+      </c>
+      <c r="D14">
+        <v>5</v>
+      </c>
+      <c r="E14">
+        <v>7</v>
+      </c>
+      <c r="F14">
+        <v>627</v>
+      </c>
+      <c r="G14">
+        <v>2569</v>
+      </c>
+      <c r="H14">
+        <v>3</v>
+      </c>
+      <c r="I14">
+        <v>311</v>
+      </c>
+      <c r="J14">
+        <v>319</v>
+      </c>
+      <c r="L14" s="1"/>
+      <c r="O14" s="1"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>442</v>
+      </c>
+      <c r="B15">
+        <v>5</v>
+      </c>
+      <c r="C15">
+        <v>5</v>
+      </c>
+      <c r="D15">
+        <v>5</v>
+      </c>
+      <c r="E15">
+        <v>7</v>
+      </c>
+      <c r="F15">
+        <v>712</v>
+      </c>
+      <c r="G15">
+        <v>3009</v>
+      </c>
+      <c r="H15">
+        <v>3</v>
+      </c>
+      <c r="I15">
+        <v>392</v>
+      </c>
+      <c r="J15">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>509</v>
+      </c>
+      <c r="B16">
+        <v>5</v>
+      </c>
+      <c r="C16">
+        <v>6</v>
+      </c>
+      <c r="D16">
+        <v>5</v>
+      </c>
+      <c r="E16">
+        <v>7</v>
+      </c>
+      <c r="F16">
+        <v>822</v>
+      </c>
+      <c r="G16">
+        <v>3429</v>
+      </c>
+      <c r="H16">
+        <v>3</v>
+      </c>
+      <c r="I16">
+        <v>434</v>
+      </c>
+      <c r="J16">
+        <v>421</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>575</v>
+      </c>
+      <c r="B17">
+        <v>6</v>
+      </c>
+      <c r="C17">
+        <v>6</v>
+      </c>
+      <c r="D17">
+        <v>5</v>
+      </c>
+      <c r="E17">
+        <v>7</v>
+      </c>
+      <c r="F17">
+        <v>944</v>
+      </c>
+      <c r="G17">
+        <v>3946</v>
+      </c>
+      <c r="H17">
+        <v>3</v>
+      </c>
+      <c r="I17">
+        <v>502</v>
+      </c>
+      <c r="J17">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>654</v>
+      </c>
+      <c r="B18">
+        <v>6</v>
+      </c>
+      <c r="C18">
+        <v>6</v>
+      </c>
+      <c r="D18">
+        <v>6</v>
+      </c>
+      <c r="E18">
+        <v>8</v>
+      </c>
+      <c r="F18">
+        <v>1062</v>
+      </c>
+      <c r="G18">
+        <v>4463</v>
+      </c>
+      <c r="H18">
+        <v>4</v>
+      </c>
+      <c r="I18">
+        <v>534</v>
+      </c>
+      <c r="J18">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>737</v>
+      </c>
+      <c r="B19">
+        <v>6</v>
+      </c>
+      <c r="C19">
+        <v>8</v>
+      </c>
+      <c r="D19">
+        <v>5</v>
+      </c>
+      <c r="E19">
+        <v>8</v>
+      </c>
+      <c r="F19">
+        <v>1188</v>
+      </c>
+      <c r="G19">
+        <v>5012</v>
+      </c>
+      <c r="H19">
+        <v>4</v>
+      </c>
+      <c r="I19">
+        <v>623</v>
+      </c>
+      <c r="J19">
+        <v>629</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>847</v>
+      </c>
+      <c r="B20">
+        <v>7</v>
+      </c>
+      <c r="C20">
+        <v>9</v>
+      </c>
+      <c r="D20">
+        <v>6</v>
+      </c>
+      <c r="E20">
+        <v>11</v>
+      </c>
+      <c r="F20">
+        <v>1322</v>
+      </c>
+      <c r="G20">
+        <v>5554</v>
+      </c>
+      <c r="H20">
+        <v>4</v>
+      </c>
+      <c r="I20">
+        <v>694</v>
+      </c>
+      <c r="J20">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>922</v>
+      </c>
+      <c r="B21">
+        <v>8</v>
+      </c>
+      <c r="C21">
+        <v>9</v>
+      </c>
+      <c r="D21">
+        <v>7</v>
+      </c>
+      <c r="E21">
+        <v>10</v>
+      </c>
+      <c r="F21">
+        <v>1479</v>
+      </c>
+      <c r="G21">
+        <v>6892</v>
+      </c>
+      <c r="H21">
+        <v>4</v>
+      </c>
+      <c r="I21">
+        <v>838</v>
+      </c>
+      <c r="J21">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="L22" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A03C4F7-C884-4CF3-883D-5363760C0851}">
+  <dimension ref="A1:P21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>3</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>4</v>
+      </c>
+      <c r="G2">
+        <v>14</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>14</v>
+      </c>
+      <c r="B3">
         <v>1</v>
       </c>
       <c r="C3">
@@ -527,21 +1227,706 @@
         <v>14</v>
       </c>
       <c r="G3">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H3">
-        <v>44</v>
+        <v>0</v>
       </c>
       <c r="I3">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>32</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>35</v>
+      </c>
+      <c r="G4">
+        <v>129</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>55</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>59</v>
+      </c>
+      <c r="G5">
+        <v>218</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>89</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6">
+        <v>90</v>
+      </c>
+      <c r="G6">
+        <v>348</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>126</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7">
+        <v>131</v>
+      </c>
+      <c r="G7">
+        <v>509</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>177</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8">
+        <v>3</v>
+      </c>
+      <c r="F8">
+        <v>177</v>
+      </c>
+      <c r="G8">
+        <v>708</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>231</v>
+      </c>
+      <c r="B9">
+        <v>3</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9">
+        <v>3</v>
+      </c>
+      <c r="F9">
+        <v>231</v>
+      </c>
+      <c r="G9">
+        <v>940</v>
+      </c>
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>289</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10">
+        <v>3</v>
+      </c>
+      <c r="D10">
+        <v>2</v>
+      </c>
+      <c r="E10">
+        <v>4</v>
+      </c>
+      <c r="F10">
+        <v>293</v>
+      </c>
+      <c r="G10">
+        <v>1216</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>364</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
+      </c>
+      <c r="C11">
+        <v>3</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11">
+        <v>5</v>
+      </c>
+      <c r="F11">
+        <v>399</v>
+      </c>
+      <c r="G11">
+        <v>1716</v>
+      </c>
+      <c r="H11">
+        <v>1</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11" s="2"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>513</v>
+      </c>
+      <c r="B12">
+        <v>4</v>
+      </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
+      <c r="D12">
+        <v>3</v>
+      </c>
+      <c r="E12">
+        <v>5</v>
+      </c>
+      <c r="F12">
+        <v>552</v>
+      </c>
+      <c r="G12">
+        <v>2190</v>
+      </c>
+      <c r="H12">
+        <v>2</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>606</v>
+      </c>
+      <c r="B13">
+        <v>4</v>
+      </c>
+      <c r="C13">
+        <v>4</v>
+      </c>
+      <c r="D13">
+        <v>3</v>
+      </c>
+      <c r="E13">
+        <v>6</v>
+      </c>
+      <c r="F13">
+        <v>577</v>
+      </c>
+      <c r="G13">
+        <v>2512</v>
+      </c>
+      <c r="H13">
+        <v>2</v>
+      </c>
+      <c r="I13">
+        <v>1</v>
+      </c>
+      <c r="J13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>734</v>
+      </c>
+      <c r="B14">
+        <v>6</v>
+      </c>
+      <c r="C14">
+        <v>3</v>
+      </c>
+      <c r="D14">
+        <v>6</v>
+      </c>
+      <c r="E14">
+        <v>10</v>
+      </c>
+      <c r="F14">
+        <v>824</v>
+      </c>
+      <c r="G14">
+        <v>2927</v>
+      </c>
+      <c r="H14">
+        <v>1</v>
+      </c>
+      <c r="I14">
+        <v>1</v>
+      </c>
+      <c r="J14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>860</v>
+      </c>
+      <c r="B15">
+        <v>5</v>
+      </c>
+      <c r="C15">
+        <v>6</v>
+      </c>
+      <c r="D15">
+        <v>5</v>
+      </c>
+      <c r="E15">
+        <v>9</v>
+      </c>
+      <c r="F15">
+        <v>932</v>
+      </c>
+      <c r="G15">
+        <v>3444</v>
+      </c>
+      <c r="H15">
+        <v>2</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>1</v>
+      </c>
+      <c r="P15" s="1"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>960</v>
+      </c>
+      <c r="B16">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="C16">
+        <v>6</v>
+      </c>
+      <c r="D16">
+        <v>5</v>
+      </c>
+      <c r="E16">
+        <v>12</v>
+      </c>
+      <c r="F16">
+        <v>997</v>
+      </c>
+      <c r="G16">
+        <v>3922</v>
+      </c>
+      <c r="H16">
+        <v>2</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>1026</v>
+      </c>
+      <c r="B17">
+        <v>6</v>
+      </c>
+      <c r="C17">
+        <v>4</v>
+      </c>
+      <c r="D17">
+        <v>5</v>
+      </c>
+      <c r="E17">
+        <v>7</v>
+      </c>
+      <c r="F17">
+        <v>1023</v>
+      </c>
+      <c r="G17">
+        <v>4168</v>
+      </c>
+      <c r="H17">
+        <v>2</v>
+      </c>
+      <c r="I17">
+        <v>0</v>
+      </c>
+      <c r="J17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>1056</v>
+      </c>
+      <c r="B18">
+        <v>6</v>
+      </c>
+      <c r="C18">
+        <v>5</v>
+      </c>
+      <c r="D18">
+        <v>5</v>
+      </c>
+      <c r="E18">
+        <v>8</v>
+      </c>
+      <c r="F18">
+        <v>1047</v>
+      </c>
+      <c r="G18">
+        <v>4457</v>
+      </c>
+      <c r="H18">
+        <v>2</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>1190</v>
+      </c>
+      <c r="B19">
+        <v>6</v>
+      </c>
+      <c r="C19">
+        <v>6</v>
+      </c>
+      <c r="D19">
+        <v>5</v>
+      </c>
+      <c r="E19">
+        <v>9</v>
+      </c>
+      <c r="F19">
+        <v>1153</v>
+      </c>
+      <c r="G19">
+        <v>5018</v>
+      </c>
+      <c r="H19">
+        <v>2</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>1</v>
+      </c>
+      <c r="M19" s="1"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>1333</v>
+      </c>
+      <c r="B20">
+        <v>6</v>
+      </c>
+      <c r="C20">
+        <v>6</v>
+      </c>
+      <c r="D20">
+        <v>5</v>
+      </c>
+      <c r="E20">
+        <v>10</v>
+      </c>
+      <c r="F20">
+        <v>1302</v>
+      </c>
+      <c r="G20">
+        <v>5602</v>
+      </c>
+      <c r="H20">
+        <v>3</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>1453</v>
+      </c>
+      <c r="B21">
+        <v>7</v>
+      </c>
+      <c r="C21">
+        <v>6</v>
+      </c>
+      <c r="D21">
+        <v>5</v>
+      </c>
+      <c r="E21">
+        <v>10</v>
+      </c>
+      <c r="F21">
+        <v>1435</v>
+      </c>
+      <c r="G21">
+        <v>6155</v>
+      </c>
+      <c r="H21">
+        <v>2</v>
+      </c>
+      <c r="I21">
+        <v>1</v>
+      </c>
+      <c r="J21">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C4F669A-5226-448C-A248-D88E4337FCEC}">
+  <dimension ref="A1:M21"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>3</v>
+      </c>
+      <c r="G2">
+        <v>13</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>1</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>0</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>1</v>
+      </c>
+      <c r="F3">
+        <v>14</v>
+      </c>
+      <c r="G3">
+        <v>49</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
+      <c r="I3">
+        <v>3</v>
+      </c>
+      <c r="J3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -559,85 +1944,85 @@
         <v>32</v>
       </c>
       <c r="G4">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="H4">
-        <v>66</v>
+        <v>1</v>
       </c>
       <c r="I4">
+        <v>8</v>
+      </c>
+      <c r="J4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5">
+        <v>60</v>
+      </c>
+      <c r="G5">
+        <v>212</v>
+      </c>
+      <c r="H5">
+        <v>1</v>
+      </c>
+      <c r="I5">
+        <v>14</v>
+      </c>
+      <c r="J5">
         <v>15</v>
       </c>
-      <c r="J4">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>35</v>
-      </c>
-      <c r="B5">
-        <v>1</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>1</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
-      <c r="F5">
-        <v>56</v>
-      </c>
-      <c r="G5">
-        <v>217</v>
-      </c>
-      <c r="H5">
-        <v>98</v>
-      </c>
-      <c r="I5">
-        <v>29</v>
-      </c>
-      <c r="J5">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>57</v>
+        <v>1</v>
       </c>
       <c r="B6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6">
         <v>2</v>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F6">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G6">
-        <v>355</v>
+        <v>338</v>
       </c>
       <c r="H6">
-        <v>105</v>
+        <v>2</v>
       </c>
       <c r="I6">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="J6">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>87</v>
+        <v>2</v>
       </c>
       <c r="B7">
         <v>2</v>
@@ -649,33 +2034,33 @@
         <v>2</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F7">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="G7">
-        <v>510</v>
+        <v>500</v>
       </c>
       <c r="H7">
-        <v>192</v>
+        <v>2</v>
       </c>
       <c r="I7">
-        <v>64</v>
+        <v>36</v>
       </c>
       <c r="J7">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>110</v>
+        <v>2</v>
       </c>
       <c r="B8">
         <v>2</v>
       </c>
       <c r="C8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D8">
         <v>2</v>
@@ -684,56 +2069,56 @@
         <v>3</v>
       </c>
       <c r="F8">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="G8">
-        <v>707</v>
+        <v>698</v>
       </c>
       <c r="H8">
-        <v>153</v>
+        <v>2</v>
       </c>
       <c r="I8">
-        <v>97</v>
+        <v>46</v>
       </c>
       <c r="J8">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>144</v>
+        <v>3</v>
       </c>
       <c r="B9">
         <v>3</v>
       </c>
       <c r="C9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D9">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E9">
         <v>4</v>
       </c>
       <c r="F9">
-        <v>253</v>
+        <v>232</v>
       </c>
       <c r="G9">
-        <v>939</v>
+        <v>919</v>
       </c>
       <c r="H9">
-        <v>177</v>
+        <v>3</v>
       </c>
       <c r="I9">
-        <v>127</v>
+        <v>63</v>
       </c>
       <c r="J9">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>184</v>
+        <v>3</v>
       </c>
       <c r="B10">
         <v>3</v>
@@ -742,30 +2127,30 @@
         <v>3</v>
       </c>
       <c r="D10">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E10">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F10">
-        <v>295</v>
+        <v>306</v>
       </c>
       <c r="G10">
-        <v>1194</v>
+        <v>1207</v>
       </c>
       <c r="H10">
-        <v>221</v>
+        <v>2</v>
       </c>
       <c r="I10">
-        <v>156</v>
+        <v>81</v>
       </c>
       <c r="J10">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>244</v>
+        <v>3</v>
       </c>
       <c r="B11">
         <v>3</v>
@@ -774,62 +2159,62 @@
         <v>4</v>
       </c>
       <c r="D11">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E11">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F11">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G11">
-        <v>1501</v>
+        <v>1476</v>
       </c>
       <c r="H11">
-        <v>238</v>
+        <v>4</v>
       </c>
       <c r="I11">
-        <v>192</v>
+        <v>93</v>
       </c>
       <c r="J11">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>284</v>
+        <v>3</v>
       </c>
       <c r="B12">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C12">
         <v>4</v>
       </c>
       <c r="D12">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E12">
         <v>5</v>
       </c>
       <c r="F12">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="G12">
         <v>1808</v>
       </c>
       <c r="H12">
-        <v>306</v>
+        <v>3</v>
       </c>
       <c r="I12">
-        <v>242</v>
+        <v>120</v>
       </c>
       <c r="J12">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>326</v>
+        <v>3</v>
       </c>
       <c r="B13">
         <v>5</v>
@@ -838,126 +2223,127 @@
         <v>4</v>
       </c>
       <c r="D13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E13">
         <v>5</v>
       </c>
       <c r="F13">
-        <v>518</v>
+        <v>534</v>
       </c>
       <c r="G13">
-        <v>2156</v>
+        <v>2126</v>
       </c>
       <c r="H13">
-        <v>341</v>
+        <v>4</v>
       </c>
       <c r="I13">
-        <v>268</v>
+        <v>133</v>
       </c>
       <c r="J13">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>389</v>
+        <v>3</v>
       </c>
       <c r="B14">
         <v>5</v>
       </c>
       <c r="C14">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E14">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F14">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="G14">
-        <v>2533</v>
+        <v>2600</v>
       </c>
       <c r="H14">
-        <v>446</v>
+        <v>5</v>
       </c>
       <c r="I14">
-        <v>315</v>
+        <v>157</v>
       </c>
       <c r="J14">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>449</v>
+        <v>4</v>
       </c>
       <c r="B15">
         <v>5</v>
       </c>
       <c r="C15">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D15">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E15">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F15">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="G15">
-        <v>2995</v>
+        <v>2981</v>
       </c>
       <c r="H15">
-        <v>380</v>
+        <v>5</v>
       </c>
       <c r="I15">
-        <v>380</v>
+        <v>194</v>
       </c>
       <c r="J15">
-        <v>369</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+        <v>196</v>
+      </c>
+      <c r="M15" s="1"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>518</v>
+        <v>4</v>
       </c>
       <c r="B16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C16">
         <v>6</v>
       </c>
       <c r="D16">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E16">
         <v>8</v>
       </c>
       <c r="F16">
-        <v>824</v>
+        <v>821</v>
       </c>
       <c r="G16">
-        <v>3410</v>
+        <v>3435</v>
       </c>
       <c r="H16">
-        <v>371</v>
+        <v>6</v>
       </c>
       <c r="I16">
-        <v>443</v>
+        <v>216</v>
       </c>
       <c r="J16">
-        <v>421</v>
+        <v>215</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>592</v>
+        <v>5</v>
       </c>
       <c r="B17">
         <v>6</v>
@@ -966,132 +2352,132 @@
         <v>6</v>
       </c>
       <c r="D17">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E17">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F17">
-        <v>940</v>
+        <v>932</v>
       </c>
       <c r="G17">
-        <v>3889</v>
+        <v>3890</v>
       </c>
       <c r="H17">
-        <v>450</v>
+        <v>6</v>
       </c>
       <c r="I17">
-        <v>487</v>
+        <v>246</v>
       </c>
       <c r="J17">
-        <v>480</v>
+        <v>248</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>665</v>
+        <v>5</v>
       </c>
       <c r="B18">
         <v>6</v>
       </c>
       <c r="C18">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E18">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F18">
-        <v>1070</v>
+        <v>1061</v>
       </c>
       <c r="G18">
-        <v>4510</v>
+        <v>4467</v>
       </c>
       <c r="H18">
-        <v>612</v>
+        <v>6</v>
       </c>
       <c r="I18">
-        <v>564</v>
+        <v>287</v>
       </c>
       <c r="J18">
-        <v>554</v>
+        <v>289</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>739</v>
+        <v>5</v>
       </c>
       <c r="B19">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C19">
         <v>8</v>
       </c>
       <c r="D19">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E19">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F19">
-        <v>1189</v>
+        <v>1185</v>
       </c>
       <c r="G19">
-        <v>4944</v>
+        <v>4957</v>
       </c>
       <c r="H19">
-        <v>572</v>
+        <v>8</v>
       </c>
       <c r="I19">
-        <v>615</v>
+        <v>333</v>
       </c>
       <c r="J19">
-        <v>626</v>
+        <v>323</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>1046</v>
+        <v>6</v>
       </c>
       <c r="B20">
+        <v>6</v>
+      </c>
+      <c r="C20">
+        <v>9</v>
+      </c>
+      <c r="D20">
+        <v>7</v>
+      </c>
+      <c r="E20">
         <v>10</v>
       </c>
-      <c r="C20">
-        <v>8</v>
-      </c>
-      <c r="D20">
-        <v>6</v>
-      </c>
-      <c r="E20">
-        <v>12</v>
-      </c>
       <c r="F20">
-        <v>1542</v>
+        <v>1323</v>
       </c>
       <c r="G20">
-        <v>6434</v>
+        <v>5547</v>
       </c>
       <c r="H20">
-        <v>731</v>
+        <v>7</v>
       </c>
       <c r="I20">
-        <v>792</v>
+        <v>350</v>
       </c>
       <c r="J20">
-        <v>775</v>
+        <v>356</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>1070</v>
+        <v>6</v>
       </c>
       <c r="B21">
         <v>7</v>
       </c>
       <c r="C21">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D21">
         <v>7</v>
@@ -1100,19 +2486,19 @@
         <v>11</v>
       </c>
       <c r="F21">
-        <v>1833</v>
+        <v>1480</v>
       </c>
       <c r="G21">
-        <v>6569</v>
+        <v>6584</v>
       </c>
       <c r="H21">
-        <v>538</v>
+        <v>12</v>
       </c>
       <c r="I21">
-        <v>894</v>
+        <v>543</v>
       </c>
       <c r="J21">
-        <v>848</v>
+        <v>576</v>
       </c>
     </row>
   </sheetData>

</xml_diff>